<commit_message>
Add CORS, static asset serving, and txid primary key support
- Add CORS middleware so web app can call the API cross-origin
- Serve Expo app assets folder as static files at /assets
- Support txid as fallback primary key in sheetToRows (dashboard sheet)
- Update database.xlsx with dashboard sheet data

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/database.xlsx
+++ b/data/database.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10817"/>
-  <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD04E798-FF56-C142-B406-874CB0518ACA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="4360" yWindow="660" windowWidth="30200" windowHeight="20160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680"/>
   </bookViews>
   <sheets>
-    <sheet name="products" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="products" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="dashboard" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="134">
   <si>
     <t>id</t>
   </si>
@@ -30,19 +30,406 @@
   </si>
   <si>
     <t>my first prod</t>
+  </si>
+  <si>
+    <t>txid</t>
+  </si>
+  <si>
+    <t>Dashcaption</t>
+  </si>
+  <si>
+    <t>dash_image</t>
+  </si>
+  <si>
+    <t>appviewsheet</t>
+  </si>
+  <si>
+    <t>parentview</t>
+  </si>
+  <si>
+    <t>userrole</t>
+  </si>
+  <si>
+    <t>screen_order</t>
+  </si>
+  <si>
+    <t>Rating</t>
+  </si>
+  <si>
+    <t>dashboard_Images/80486473.image.090130.png</t>
+  </si>
+  <si>
+    <t>Student Rating</t>
+  </si>
+  <si>
+    <t>Students</t>
+  </si>
+  <si>
+    <t>Course</t>
+  </si>
+  <si>
+    <t>dashboard_Images/Course.image.013811.png</t>
+  </si>
+  <si>
+    <t>Courses View</t>
+  </si>
+  <si>
+    <t>Time Table</t>
+  </si>
+  <si>
+    <t>dashboard_Images/13d34056.image.035329.png</t>
+  </si>
+  <si>
+    <t>CourseTimeTableView</t>
+  </si>
+  <si>
+    <t>Observation Qn</t>
+  </si>
+  <si>
+    <t>dashboard_Images/question.png</t>
+  </si>
+  <si>
+    <t>Obeservation Qns</t>
+  </si>
+  <si>
+    <t>Fee Summary</t>
+  </si>
+  <si>
+    <t>dashboard_Images/Student Fees Summary.image.013944.png</t>
+  </si>
+  <si>
+    <t>Student Fee Summary</t>
+  </si>
+  <si>
+    <t>Admin</t>
+  </si>
+  <si>
+    <t>Expense</t>
+  </si>
+  <si>
+    <t>dashboard_Images/Expense.image.013510.png</t>
+  </si>
+  <si>
+    <t>Expenses View</t>
+  </si>
+  <si>
+    <t>Finance</t>
+  </si>
+  <si>
+    <t>Staff Salary</t>
+  </si>
+  <si>
+    <t>dashboard_Images/Staff Salary.image.013547.png</t>
+  </si>
+  <si>
+    <t>SalarySetup</t>
+  </si>
+  <si>
+    <t>dashboard_Images/Student Fee.image.013619.png</t>
+  </si>
+  <si>
+    <t>Student Fee</t>
+  </si>
+  <si>
+    <t>Class Fee Summary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pending Fees </t>
+  </si>
+  <si>
+    <t>dashboard_Images/df.image.080223.png</t>
+  </si>
+  <si>
+    <t>Student Fee Pending</t>
+  </si>
+  <si>
+    <t>Monthly Fee Summary</t>
+  </si>
+  <si>
+    <t>dashboard_Images/Class Fees Summary.image.014040.png</t>
+  </si>
+  <si>
+    <t>Financial Summary</t>
+  </si>
+  <si>
+    <t>dashboard_Images/Financial Summary.image.014121.png</t>
+  </si>
+  <si>
+    <t>Finance Summary</t>
+  </si>
+  <si>
+    <t>Expeses Summary</t>
+  </si>
+  <si>
+    <t>dashboard_Images/Expeses Summary.image.014857.png</t>
+  </si>
+  <si>
+    <t>ExpeseSummery_Rpt</t>
+  </si>
+  <si>
+    <t>Manage</t>
+  </si>
+  <si>
+    <t>dashboard_Images/7ee0dee0.dash_image.060625.png</t>
+  </si>
+  <si>
+    <t>Student View</t>
+  </si>
+  <si>
+    <t>Assignments</t>
+  </si>
+  <si>
+    <t>dashboard_Images/80a95210.dash_image.065304.png</t>
+  </si>
+  <si>
+    <t>Student Activity</t>
+  </si>
+  <si>
+    <t>Attendance</t>
+  </si>
+  <si>
+    <t>dashboard_Images/df.image.111601.png</t>
+  </si>
+  <si>
+    <t>student att dash</t>
+  </si>
+  <si>
+    <t>Leave</t>
+  </si>
+  <si>
+    <t>dashboard_Images/Student Leave.image.0133262.png</t>
+  </si>
+  <si>
+    <t>Student leave log</t>
+  </si>
+  <si>
+    <t>dashboard_Images/f23b0784.dash_image.091042.png</t>
+  </si>
+  <si>
+    <t>Collect Fee</t>
+  </si>
+  <si>
+    <t>dashboard_Images/collectFee.png</t>
+  </si>
+  <si>
+    <t>st_fee_Form</t>
+  </si>
+  <si>
+    <t>Fee Pending</t>
+  </si>
+  <si>
+    <t>dashboard_Images/question_st.png</t>
+  </si>
+  <si>
+    <t>Obeservations_st</t>
+  </si>
+  <si>
+    <t>Progress Card</t>
+  </si>
+  <si>
+    <t>dashboard_Images/da6bd0ad.dash_image.092247.png</t>
+  </si>
+  <si>
+    <t>Student Marks</t>
+  </si>
+  <si>
+    <t>dashboard_Images/dd.image.082709.png</t>
+  </si>
+  <si>
+    <t>Teachers View</t>
+  </si>
+  <si>
+    <t>Teachers</t>
+  </si>
+  <si>
+    <t>Activity</t>
+  </si>
+  <si>
+    <t>dashboard_Images/a0cd3bd7.image.041908.png</t>
+  </si>
+  <si>
+    <t>Teacher Activity</t>
+  </si>
+  <si>
+    <t>Salary</t>
+  </si>
+  <si>
+    <t>dashboard_Images/f4dbb49d.image.035921.png</t>
+  </si>
+  <si>
+    <t>dashboard_Images/abeebe66.image.040651.png</t>
+  </si>
+  <si>
+    <t>TeacherAttDash</t>
+  </si>
+  <si>
+    <t>dashboard_Images/fac3c273.image.035751.png</t>
+  </si>
+  <si>
+    <t>Teacher leave log</t>
+  </si>
+  <si>
+    <t>Schedule</t>
+  </si>
+  <si>
+    <t>Teacher Schedule</t>
+  </si>
+  <si>
+    <t>Teacher Dash View</t>
+  </si>
+  <si>
+    <t>Home</t>
+  </si>
+  <si>
+    <t>Courses</t>
+  </si>
+  <si>
+    <t>dashboard_Images/dss.image.082849.png</t>
+  </si>
+  <si>
+    <t>Course Dash</t>
+  </si>
+  <si>
+    <t>My Schedule</t>
+  </si>
+  <si>
+    <t>dashboard_Images/sd.image.082559.png</t>
+  </si>
+  <si>
+    <t>TeacherTimeTable</t>
+  </si>
+  <si>
+    <t>dashboard_Images/Students.image.012707.png</t>
+  </si>
+  <si>
+    <t>Student Dash View</t>
+  </si>
+  <si>
+    <t>dashboard_Images/ff.image.082511.png</t>
+  </si>
+  <si>
+    <t>Finance Dash</t>
+  </si>
+  <si>
+    <t>My Task</t>
+  </si>
+  <si>
+    <t>dashboard_Images/df.image.081653.png</t>
+  </si>
+  <si>
+    <t>TODO</t>
+  </si>
+  <si>
+    <t>Course Attendance</t>
+  </si>
+  <si>
+    <t>dashboard_Images/Course Attendance.image.060791.png</t>
+  </si>
+  <si>
+    <t>Student attendance by Course</t>
+  </si>
+  <si>
+    <t>Scan Attendance QR</t>
+  </si>
+  <si>
+    <t>dashboard_Images/ss.image.081803.png</t>
+  </si>
+  <si>
+    <t>ScanMyAttendance</t>
+  </si>
+  <si>
+    <t>Class Diary</t>
+  </si>
+  <si>
+    <t>dashboard_Images/1b10b898.dash_image.092006.png</t>
+  </si>
+  <si>
+    <t>ClassDiary</t>
+  </si>
+  <si>
+    <t>Holidays</t>
+  </si>
+  <si>
+    <t>dashboard_Images/sdsa.image.082204.png</t>
+  </si>
+  <si>
+    <t>Assingment</t>
+  </si>
+  <si>
+    <t>Class Assingment</t>
+  </si>
+  <si>
+    <t>My Students Marks</t>
+  </si>
+  <si>
+    <t>dashboard_Images/5fb3e3cc.image.042406.png</t>
+  </si>
+  <si>
+    <t>Teacher Student Marks</t>
+  </si>
+  <si>
+    <t>Student Diary</t>
+  </si>
+  <si>
+    <t>dashboard_Images/8df8cea3.image.084606.png</t>
+  </si>
+  <si>
+    <t>Teacher Rating</t>
+  </si>
+  <si>
+    <t>Parent Note</t>
+  </si>
+  <si>
+    <t>dashboard_Images/661276c6.dash_image.171435.png</t>
+  </si>
+  <si>
+    <t>FeedBack/Complaints</t>
+  </si>
+  <si>
+    <t>dashboard_Images/f4e38ab5.dash_image.064659.png</t>
+  </si>
+  <si>
+    <t>FeedBack</t>
+  </si>
+  <si>
+    <t>Enquiries</t>
+  </si>
+  <si>
+    <t>dashboard_Images/3eb53695.dash_image.092144.png</t>
+  </si>
+  <si>
+    <t>Handbook</t>
+  </si>
+  <si>
+    <t>dashboard_images/502d45f4.dash_image.182747.png</t>
+  </si>
+  <si>
+    <t>Meeting Notes</t>
+  </si>
+  <si>
+    <t>dashboard_Images/Meetin_Notes.png</t>
+  </si>
+  <si>
+    <t>Health Data</t>
+  </si>
+  <si>
+    <t>dashboard_Images/StudentMedical.png</t>
+  </si>
+  <si>
+    <t>Health_Record</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -405,11 +792,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.83203125"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -423,7 +810,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>11</v>
       </c>
@@ -439,6 +826,994 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G49"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>80486473</v>
+      </c>
+      <c r="B2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>80486474</v>
+      </c>
+      <c r="B3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>80486475</v>
+      </c>
+      <c r="B4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>80186485</v>
+      </c>
+      <c r="B5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D5" t="s">
+        <v>24</v>
+      </c>
+      <c r="E5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>80486079</v>
+      </c>
+      <c r="B6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" t="s">
+        <v>27</v>
+      </c>
+      <c r="E6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F6" t="s">
+        <v>28</v>
+      </c>
+      <c r="G6">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>80486476</v>
+      </c>
+      <c r="B7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" t="s">
+        <v>30</v>
+      </c>
+      <c r="D7" t="s">
+        <v>31</v>
+      </c>
+      <c r="E7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>80486477</v>
+      </c>
+      <c r="B8" t="s">
+        <v>33</v>
+      </c>
+      <c r="C8" t="s">
+        <v>34</v>
+      </c>
+      <c r="D8" t="s">
+        <v>35</v>
+      </c>
+      <c r="E8" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>80486478</v>
+      </c>
+      <c r="B9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D9" t="s">
+        <v>37</v>
+      </c>
+      <c r="E9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>80486479</v>
+      </c>
+      <c r="B10" t="s">
+        <v>38</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10" t="s">
+        <v>27</v>
+      </c>
+      <c r="E10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>80486480</v>
+      </c>
+      <c r="B11" t="s">
+        <v>39</v>
+      </c>
+      <c r="C11" t="s">
+        <v>40</v>
+      </c>
+      <c r="D11" t="s">
+        <v>41</v>
+      </c>
+      <c r="E11" t="s">
+        <v>32</v>
+      </c>
+      <c r="F11" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>80486481</v>
+      </c>
+      <c r="B12" t="s">
+        <v>42</v>
+      </c>
+      <c r="C12" t="s">
+        <v>43</v>
+      </c>
+      <c r="D12" t="s">
+        <v>38</v>
+      </c>
+      <c r="E12" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>80486482</v>
+      </c>
+      <c r="B13" t="s">
+        <v>44</v>
+      </c>
+      <c r="C13" t="s">
+        <v>45</v>
+      </c>
+      <c r="D13" t="s">
+        <v>46</v>
+      </c>
+      <c r="E13" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>80486483</v>
+      </c>
+      <c r="B14" t="s">
+        <v>47</v>
+      </c>
+      <c r="C14" t="s">
+        <v>48</v>
+      </c>
+      <c r="D14" t="s">
+        <v>49</v>
+      </c>
+      <c r="E14" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>80486484</v>
+      </c>
+      <c r="B15" t="s">
+        <v>50</v>
+      </c>
+      <c r="C15" t="s">
+        <v>51</v>
+      </c>
+      <c r="D15" t="s">
+        <v>52</v>
+      </c>
+      <c r="E15" t="s">
+        <v>15</v>
+      </c>
+      <c r="G15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>80486485</v>
+      </c>
+      <c r="B16" t="s">
+        <v>53</v>
+      </c>
+      <c r="C16" t="s">
+        <v>54</v>
+      </c>
+      <c r="D16" t="s">
+        <v>55</v>
+      </c>
+      <c r="E16" t="s">
+        <v>15</v>
+      </c>
+      <c r="G16">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>80486486</v>
+      </c>
+      <c r="B17" t="s">
+        <v>56</v>
+      </c>
+      <c r="C17" t="s">
+        <v>57</v>
+      </c>
+      <c r="D17" t="s">
+        <v>58</v>
+      </c>
+      <c r="E17" t="s">
+        <v>15</v>
+      </c>
+      <c r="G17">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>80486487</v>
+      </c>
+      <c r="B18" t="s">
+        <v>59</v>
+      </c>
+      <c r="C18" t="s">
+        <v>60</v>
+      </c>
+      <c r="D18" t="s">
+        <v>61</v>
+      </c>
+      <c r="E18" t="s">
+        <v>15</v>
+      </c>
+      <c r="G18">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>80486488</v>
+      </c>
+      <c r="B19" t="s">
+        <v>25</v>
+      </c>
+      <c r="C19" t="s">
+        <v>62</v>
+      </c>
+      <c r="D19" t="s">
+        <v>37</v>
+      </c>
+      <c r="E19" t="s">
+        <v>15</v>
+      </c>
+      <c r="F19" t="s">
+        <v>28</v>
+      </c>
+      <c r="G19">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>804864891</v>
+      </c>
+      <c r="B20" t="s">
+        <v>63</v>
+      </c>
+      <c r="C20" t="s">
+        <v>64</v>
+      </c>
+      <c r="D20" t="s">
+        <v>65</v>
+      </c>
+      <c r="E20" t="s">
+        <v>15</v>
+      </c>
+      <c r="F20" t="s">
+        <v>28</v>
+      </c>
+      <c r="G20">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>80486489</v>
+      </c>
+      <c r="B21" t="s">
+        <v>66</v>
+      </c>
+      <c r="C21" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21" t="s">
+        <v>41</v>
+      </c>
+      <c r="E21" t="s">
+        <v>15</v>
+      </c>
+      <c r="F21" t="s">
+        <v>28</v>
+      </c>
+      <c r="G21">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>80286485</v>
+      </c>
+      <c r="B22" t="s">
+        <v>22</v>
+      </c>
+      <c r="C22" t="s">
+        <v>67</v>
+      </c>
+      <c r="D22" t="s">
+        <v>68</v>
+      </c>
+      <c r="E22" t="s">
+        <v>15</v>
+      </c>
+      <c r="G22">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>80486490</v>
+      </c>
+      <c r="B23" t="s">
+        <v>69</v>
+      </c>
+      <c r="C23" t="s">
+        <v>70</v>
+      </c>
+      <c r="D23" t="s">
+        <v>71</v>
+      </c>
+      <c r="E23" t="s">
+        <v>15</v>
+      </c>
+      <c r="G23">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>80486491</v>
+      </c>
+      <c r="B24" t="s">
+        <v>50</v>
+      </c>
+      <c r="C24" t="s">
+        <v>72</v>
+      </c>
+      <c r="D24" t="s">
+        <v>73</v>
+      </c>
+      <c r="E24" t="s">
+        <v>74</v>
+      </c>
+      <c r="G24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>80486492</v>
+      </c>
+      <c r="B25" t="s">
+        <v>75</v>
+      </c>
+      <c r="C25" t="s">
+        <v>76</v>
+      </c>
+      <c r="D25" t="s">
+        <v>77</v>
+      </c>
+      <c r="E25" t="s">
+        <v>74</v>
+      </c>
+      <c r="G25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>80486493</v>
+      </c>
+      <c r="B26" t="s">
+        <v>78</v>
+      </c>
+      <c r="C26" t="s">
+        <v>79</v>
+      </c>
+      <c r="D26" t="s">
+        <v>33</v>
+      </c>
+      <c r="E26" t="s">
+        <v>74</v>
+      </c>
+      <c r="G26">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>80486494</v>
+      </c>
+      <c r="B27" t="s">
+        <v>56</v>
+      </c>
+      <c r="C27" t="s">
+        <v>80</v>
+      </c>
+      <c r="D27" t="s">
+        <v>81</v>
+      </c>
+      <c r="E27" t="s">
+        <v>74</v>
+      </c>
+      <c r="G27">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>80486495</v>
+      </c>
+      <c r="B28" t="s">
+        <v>59</v>
+      </c>
+      <c r="C28" t="s">
+        <v>82</v>
+      </c>
+      <c r="D28" t="s">
+        <v>83</v>
+      </c>
+      <c r="E28" t="s">
+        <v>74</v>
+      </c>
+      <c r="G28">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>80486496</v>
+      </c>
+      <c r="B29" t="s">
+        <v>84</v>
+      </c>
+      <c r="C29" t="s">
+        <v>20</v>
+      </c>
+      <c r="D29" t="s">
+        <v>85</v>
+      </c>
+      <c r="E29" t="s">
+        <v>74</v>
+      </c>
+      <c r="G29">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>80486497</v>
+      </c>
+      <c r="B30" t="s">
+        <v>74</v>
+      </c>
+      <c r="C30" t="s">
+        <v>72</v>
+      </c>
+      <c r="D30" t="s">
+        <v>86</v>
+      </c>
+      <c r="E30" t="s">
+        <v>87</v>
+      </c>
+      <c r="G30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>80486498</v>
+      </c>
+      <c r="B31" t="s">
+        <v>88</v>
+      </c>
+      <c r="C31" t="s">
+        <v>89</v>
+      </c>
+      <c r="D31" t="s">
+        <v>90</v>
+      </c>
+      <c r="E31" t="s">
+        <v>87</v>
+      </c>
+      <c r="G31">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>80486499</v>
+      </c>
+      <c r="B32" t="s">
+        <v>91</v>
+      </c>
+      <c r="C32" t="s">
+        <v>92</v>
+      </c>
+      <c r="D32" t="s">
+        <v>93</v>
+      </c>
+      <c r="E32" t="s">
+        <v>87</v>
+      </c>
+      <c r="G32">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>80486500</v>
+      </c>
+      <c r="B33" t="s">
+        <v>15</v>
+      </c>
+      <c r="C33" t="s">
+        <v>94</v>
+      </c>
+      <c r="D33" t="s">
+        <v>95</v>
+      </c>
+      <c r="E33" t="s">
+        <v>87</v>
+      </c>
+      <c r="G33">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>80486501</v>
+      </c>
+      <c r="B34" t="s">
+        <v>32</v>
+      </c>
+      <c r="C34" t="s">
+        <v>96</v>
+      </c>
+      <c r="D34" t="s">
+        <v>97</v>
+      </c>
+      <c r="E34" t="s">
+        <v>87</v>
+      </c>
+      <c r="F34" t="s">
+        <v>28</v>
+      </c>
+      <c r="G34">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35">
+        <v>80486502</v>
+      </c>
+      <c r="B35" t="s">
+        <v>98</v>
+      </c>
+      <c r="C35" t="s">
+        <v>99</v>
+      </c>
+      <c r="D35" t="s">
+        <v>100</v>
+      </c>
+      <c r="E35" t="s">
+        <v>87</v>
+      </c>
+      <c r="G35">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>80486503</v>
+      </c>
+      <c r="B36" t="s">
+        <v>101</v>
+      </c>
+      <c r="C36" t="s">
+        <v>102</v>
+      </c>
+      <c r="D36" t="s">
+        <v>103</v>
+      </c>
+      <c r="E36" t="s">
+        <v>16</v>
+      </c>
+      <c r="G36">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>80486504</v>
+      </c>
+      <c r="B37" t="s">
+        <v>104</v>
+      </c>
+      <c r="C37" t="s">
+        <v>105</v>
+      </c>
+      <c r="D37" t="s">
+        <v>106</v>
+      </c>
+      <c r="E37" t="s">
+        <v>87</v>
+      </c>
+      <c r="G37">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <v>80486505</v>
+      </c>
+      <c r="B38" t="s">
+        <v>107</v>
+      </c>
+      <c r="C38" t="s">
+        <v>108</v>
+      </c>
+      <c r="D38" t="s">
+        <v>109</v>
+      </c>
+      <c r="E38" t="s">
+        <v>16</v>
+      </c>
+      <c r="G38">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A39">
+        <v>80486506</v>
+      </c>
+      <c r="B39" t="s">
+        <v>110</v>
+      </c>
+      <c r="C39" t="s">
+        <v>111</v>
+      </c>
+      <c r="D39" t="s">
+        <v>110</v>
+      </c>
+      <c r="E39" t="s">
+        <v>87</v>
+      </c>
+      <c r="G39">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A40">
+        <v>80486507</v>
+      </c>
+      <c r="B40" t="s">
+        <v>112</v>
+      </c>
+      <c r="C40" t="s">
+        <v>54</v>
+      </c>
+      <c r="D40" t="s">
+        <v>113</v>
+      </c>
+      <c r="E40" t="s">
+        <v>16</v>
+      </c>
+      <c r="G40">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A41">
+        <v>80486508</v>
+      </c>
+      <c r="B41" t="s">
+        <v>114</v>
+      </c>
+      <c r="C41" t="s">
+        <v>115</v>
+      </c>
+      <c r="D41" t="s">
+        <v>116</v>
+      </c>
+      <c r="E41" t="s">
+        <v>74</v>
+      </c>
+      <c r="G41">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A42">
+        <v>80486509</v>
+      </c>
+      <c r="B42" t="s">
+        <v>117</v>
+      </c>
+      <c r="C42" t="s">
+        <v>108</v>
+      </c>
+      <c r="D42" t="s">
+        <v>117</v>
+      </c>
+      <c r="E42" t="s">
+        <v>15</v>
+      </c>
+      <c r="G42">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A43">
+        <v>80486510</v>
+      </c>
+      <c r="B43" t="s">
+        <v>12</v>
+      </c>
+      <c r="C43" t="s">
+        <v>118</v>
+      </c>
+      <c r="D43" t="s">
+        <v>119</v>
+      </c>
+      <c r="E43" t="s">
+        <v>74</v>
+      </c>
+      <c r="G43">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A44">
+        <v>80486511</v>
+      </c>
+      <c r="B44" t="s">
+        <v>120</v>
+      </c>
+      <c r="C44" t="s">
+        <v>121</v>
+      </c>
+      <c r="D44" t="s">
+        <v>120</v>
+      </c>
+      <c r="E44" t="s">
+        <v>15</v>
+      </c>
+      <c r="G44">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A45">
+        <v>80486512</v>
+      </c>
+      <c r="B45" t="s">
+        <v>122</v>
+      </c>
+      <c r="C45" t="s">
+        <v>123</v>
+      </c>
+      <c r="D45" t="s">
+        <v>124</v>
+      </c>
+      <c r="E45" t="s">
+        <v>74</v>
+      </c>
+      <c r="G45">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A46">
+        <v>80486513</v>
+      </c>
+      <c r="B46" t="s">
+        <v>125</v>
+      </c>
+      <c r="C46" t="s">
+        <v>126</v>
+      </c>
+      <c r="D46" t="s">
+        <v>125</v>
+      </c>
+      <c r="E46" t="s">
+        <v>87</v>
+      </c>
+      <c r="G46">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A47">
+        <v>80486514</v>
+      </c>
+      <c r="B47" t="s">
+        <v>127</v>
+      </c>
+      <c r="C47" t="s">
+        <v>128</v>
+      </c>
+      <c r="D47" t="s">
+        <v>127</v>
+      </c>
+      <c r="E47" t="s">
+        <v>74</v>
+      </c>
+      <c r="G47">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A48">
+        <v>80486515</v>
+      </c>
+      <c r="B48" t="s">
+        <v>129</v>
+      </c>
+      <c r="C48" t="s">
+        <v>130</v>
+      </c>
+      <c r="D48" t="s">
+        <v>129</v>
+      </c>
+      <c r="E48" t="s">
+        <v>87</v>
+      </c>
+      <c r="G48">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A49">
+        <v>80486516</v>
+      </c>
+      <c r="B49" t="s">
+        <v>131</v>
+      </c>
+      <c r="C49" t="s">
+        <v>132</v>
+      </c>
+      <c r="D49" t="s">
+        <v>133</v>
+      </c>
+      <c r="E49" t="s">
+        <v>15</v>
+      </c>
+      <c r="G49">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>